<commit_message>
Improve scheduling workflow and packaging
</commit_message>
<xml_diff>
--- a/人员名单/人员名单模板.xlsx
+++ b/人员名单/人员名单模板.xlsx
@@ -7,28 +7,34 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="人员名单" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Grade</t>
-  </si>
-  <si>
-    <t>Role</t>
-  </si>
-  <si>
-    <t>Campus</t>
-  </si>
-  <si>
-    <t>田宇</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="26">
+  <si>
+    <t>序号</t>
+  </si>
+  <si>
+    <t>姓名</t>
+  </si>
+  <si>
+    <t>部门</t>
+  </si>
+  <si>
+    <t>职务</t>
+  </si>
+  <si>
+    <t>专业班级</t>
+  </si>
+  <si>
+    <t>年级</t>
+  </si>
+  <si>
+    <t>校区</t>
   </si>
   <si>
     <t>张三</t>
@@ -37,28 +43,55 @@
     <t>李四</t>
   </si>
   <si>
+    <t>王五</t>
+  </si>
+  <si>
+    <t>赵六</t>
+  </si>
+  <si>
+    <t>办公室</t>
+  </si>
+  <si>
+    <t>活动部</t>
+  </si>
+  <si>
+    <t>宣传部</t>
+  </si>
+  <si>
+    <t>主任团</t>
+  </si>
+  <si>
+    <t>干事</t>
+  </si>
+  <si>
+    <t>干部</t>
+  </si>
+  <si>
+    <t>会计学2501</t>
+  </si>
+  <si>
+    <t>法学2502</t>
+  </si>
+  <si>
+    <t>计算机科学与技术2401</t>
+  </si>
+  <si>
+    <t>公共事业管理2301</t>
+  </si>
+  <si>
+    <t>大一</t>
+  </si>
+  <si>
     <t>大二</t>
   </si>
   <si>
-    <t>大一</t>
-  </si>
-  <si>
     <t>大三</t>
   </si>
   <si>
-    <t>部长</t>
-  </si>
-  <si>
-    <t>干事</t>
-  </si>
-  <si>
-    <t>主任团</t>
-  </si>
-  <si>
-    <t>南校区</t>
-  </si>
-  <si>
-    <t>北校区</t>
+    <t>旗山北校区</t>
+  </si>
+  <si>
+    <t>旗山南校区</t>
   </si>
 </sst>
 </file>
@@ -416,10 +449,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="8.7109375" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" customWidth="1"/>
+    <col min="7" max="7" width="16.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -432,47 +474,106 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>4</v>
+    <row r="2" spans="1:7">
+      <c r="A2">
+        <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>15</v>
+      </c>
+      <c r="E2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" t="s">
+        <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
-        <v>5</v>
+    <row r="3" spans="1:7">
+      <c r="A3">
+        <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="E3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
-        <v>6</v>
+    <row r="4" spans="1:7">
+      <c r="A4">
+        <v>3</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>16</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>